<commit_message>
reinicia db con nuevos datos y logica de carga, agrega metadata de carreras no incluida en archivos excel
</commit_message>
<xml_diff>
--- a/data/input/Carreras/Maestro planes.xlsx
+++ b/data/input/Carreras/Maestro planes.xlsx
@@ -15,11 +15,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={77dc95f1-3582-4c48-8b5c-d7fb3f85bd51}</author>
-    <author>tc={8dc13c32-accc-4892-b147-ce00067d393f}</author>
+    <author>tc={181ab5c2-22d5-4b00-b185-44c5ef381d4f}</author>
+    <author>tc={b18dc756-8880-40e6-b0d0-5198377e8c0f}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{77dc95f1-3582-4c48-8b5c-d7fb3f85bd51}" ref="C1">
+    <comment authorId="0" xr:uid="{181ab5c2-22d5-4b00-b185-44c5ef381d4f}" ref="C1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -28,7 +28,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{8dc13c32-accc-4892-b147-ce00067d393f}" ref="B1">
+    <comment authorId="1" xr:uid="{b18dc756-8880-40e6-b0d0-5198377e8c0f}" ref="B1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -2522,8 +2522,8 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Pablo Galliano" id="{430a3381-162b-45a9-b62e-b2de066207c9}" providerId="google-sheets"/>
-  <x18tc:person displayName="Pablo Galliano" id="{c2139c77-769b-4d34-80b9-097bd0e58129}" providerId="google-sheets"/>
+  <x18tc:person displayName="Pablo Galliano" id="{9aafbe6c-8418-4778-94fd-332a862572e8}" providerId="google-sheets"/>
+  <x18tc:person displayName="Pablo Galliano" id="{6cef9584-2210-4d48-9f5c-53852325905f}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -2723,13 +2723,13 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="C1" dT="2026-02-09T22:42:00.00" personId="{430a3381-162b-45a9-b62e-b2de066207c9}" id="{77dc95f1-3582-4c48-8b5c-d7fb3f85bd51}" done="1">
+  <x18tc:threadedComment ref="C1" dT="2026-02-09T22:42:00.00" personId="{9aafbe6c-8418-4778-94fd-332a862572e8}" id="{181ab5c2-22d5-4b00-b185-44c5ef381d4f}" done="1">
     <x18tc:text xml:space="preserve">Ver electivas IA que figuran con un 22* en el año</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="B1" dT="2026-02-07T14:38:05.00" personId="{430a3381-162b-45a9-b62e-b2de066207c9}" id="{8dc13c32-accc-4892-b147-ce00067d393f}" done="1">
+  <x18tc:threadedComment ref="B1" dT="2026-02-07T14:38:05.00" personId="{9aafbe6c-8418-4778-94fd-332a862572e8}" id="{b18dc756-8880-40e6-b0d0-5198377e8c0f}" done="1">
     <x18tc:text xml:space="preserve">codigo de plan o codigo de guarani?</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="B1" dT="2026-02-19T18:10:47.00" personId="{c2139c77-769b-4d34-80b9-097bd0e58129}" id="{fe2ae822-74cd-4047-99a3-a2c4621b6aaa}" parentId="{8dc13c32-accc-4892-b147-ce00067d393f}">
+  <x18tc:threadedComment ref="B1" dT="2026-02-19T18:10:47.00" personId="{6cef9584-2210-4d48-9f5c-53852325905f}" id="{2752d91e-772a-41f0-abd3-a2353d0a7502}" parentId="{b18dc756-8880-40e6-b0d0-5198377e8c0f}">
     <x18tc:text xml:space="preserve">use codigo de plan</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>

</xml_diff>